<commit_message>
fix: align client data contracts and join outputs
</commit_message>
<xml_diff>
--- a/docs/design/data-template/HE_Toolkit_dashboard_standard_data_template.xlsx
+++ b/docs/design/data-template/HE_Toolkit_dashboard_standard_data_template.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R66219c2fb90041bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_mapping" sheetId="2" r:id="Rcc47891b14c847e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="biology_samples" sheetId="3" r:id="R41c386d2e038441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="environmental_site_data" sheetId="4" r:id="Rbcbc33403c774870"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="flow_daily" sheetId="5" r:id="Ra60536df6526418f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="wq_long_standard" sheetId="6" r:id="R777bb188c60b4c5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rhs_summary" sheetId="7" r:id="Rbf84f1f68a354b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="joined_dataset_optional" sheetId="8" r:id="R3cec1753dedf4ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field_dictionary" sheetId="9" r:id="R0de57f5f42004c2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="validation_rules" sheetId="10" r:id="R25d9b3759a274a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb7e26ae459aa4eb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="site_mapping" sheetId="2" r:id="R176da9e678a1449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="biology_samples" sheetId="3" r:id="R1a89010476f44dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="environmental_site_data" sheetId="4" r:id="Re7b3bd20ec9745ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="flow_daily" sheetId="5" r:id="R725d3ece969c4cf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="wq_long_standard" sheetId="6" r:id="Rab8123a227824cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rhs_summary" sheetId="7" r:id="Rcaa904409fb34f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="joined_dataset_optional" sheetId="8" r:id="Rd9caea6b57f840ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field_dictionary" sheetId="9" r:id="R932ab8ac9efc41a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="validation_rules" sheetId="10" r:id="R6d71bd1110924faa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9705,15 +9705,11 @@
           <x:t xml:space="preserve">Recommended</x:t>
         </x:is>
       </x:c>
-      <x:c r="D20" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">date/text</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E20" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Start, end, duration and WQ record counts.</x:t>
-        </x:is>
+      <x:c r="D20" s="9" t="str">
+        <x:v>date/numeric</x:v>
+      </x:c>
+      <x:c r="E20" s="9" t="str">
+        <x:v>Start/end dates and inclusive duration in calendar days; WQ record counts.</x:v>
       </x:c>
       <x:c r="F20" s="9" t="inlineStr">
         <x:is>

</xml_diff>